<commit_message>
Corrida | GSF-EPRIV-INF | 2026-06-16 15:21:11.476193
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPRIV-INF_out.xlsx
+++ b/indicadores/GSF-EPRIV-INF_out.xlsx
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocupados informales en el sector privado del Gran Santa Fe</t>
+    <t xml:space="preserve">Ocupados informales en el sector privado</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -62,10 +62,10 @@
     <t xml:space="preserve">(1 0 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Código</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GSF-EPRIV-INF</t>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aglomerado Gran Santa Fe</t>
   </si>
   <si>
     <t xml:space="preserve">Regresores</t>
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/05/2026</t>
+    <t xml:space="preserve">16/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">vcorvalan</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1082,7 +1082,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.339098178992349</v>
+        <v>0.342637246779251</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1140,7 +1140,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.114987574995927</v>
+        <v>0.117400282880465</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1210,7 +1210,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.226307929213274</v>
+        <v>0.194703088502734</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1240,7 +1240,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.170596365458058</v>
+        <v>0.181311789583426</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -6601,7 +6601,7 @@
         <v>169</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0226626019595318</v>
+        <v>0.0143909663492046</v>
       </c>
     </row>
     <row r="6">
@@ -6609,7 +6609,7 @@
         <v>170</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0561963431725149</v>
+        <v>-0.0549177632913489</v>
       </c>
     </row>
     <row r="7">
@@ -6617,7 +6617,7 @@
         <v>171</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.0156912361706693</v>
+        <v>-0.00528574400128268</v>
       </c>
     </row>
     <row r="8">
@@ -6625,7 +6625,7 @@
         <v>172</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.149410474634527</v>
+        <v>0.137801449851668</v>
       </c>
     </row>
     <row r="9">
@@ -6633,7 +6633,7 @@
         <v>173</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.339098178992349</v>
+        <v>0.342637246779251</v>
       </c>
     </row>
     <row r="10">
@@ -6641,7 +6641,7 @@
         <v>174</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.127106810653067</v>
+        <v>0.133161196420219</v>
       </c>
     </row>
     <row r="11">
@@ -6649,7 +6649,7 @@
         <v>175</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.0289075947529167</v>
+        <v>0.0283701131038142</v>
       </c>
     </row>
     <row r="12">
@@ -6657,7 +6657,7 @@
         <v>176</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.185065657609698</v>
+        <v>-0.179612555020879</v>
       </c>
     </row>
     <row r="13">
@@ -6665,7 +6665,7 @@
         <v>177</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.231359469415676</v>
+        <v>-0.238445213843736</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | GSF-EPRIV-INF | 2026-06-16 15:22:59.608815
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPRIV-INF_out.xlsx
+++ b/indicadores/GSF-EPRIV-INF_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="180">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -62,16 +62,22 @@
     <t xml:space="preserve">(1 0 1)</t>
   </si>
   <si>
+    <t xml:space="preserve">Código</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GSF-EPRIV-INF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regresores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">const</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alcance</t>
   </si>
   <si>
     <t xml:space="preserve">Aglomerado Gran Santa Fe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regresores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">const</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen del correlograma</t>
@@ -1050,9 +1056,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1063,7 +1073,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1077,7 +1087,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1093,7 +1103,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1121,7 +1131,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1135,7 +1145,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1163,7 +1173,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1177,7 +1187,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1191,7 +1201,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1205,7 +1215,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1221,7 +1231,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1235,7 +1245,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1383,10 +1393,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1399,10 +1409,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1426,66 +1436,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>59.301</v>
@@ -1538,7 +1548,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>69.648</v>
@@ -1595,7 +1605,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>68.504</v>
@@ -1652,7 +1662,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>67.829</v>
@@ -1709,7 +1719,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>81.778</v>
@@ -1768,7 +1778,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>73.335</v>
@@ -1827,7 +1837,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>74.334</v>
@@ -1886,7 +1896,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>70.162</v>
@@ -1945,7 +1955,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>64.617</v>
@@ -2004,7 +2014,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>68.225</v>
@@ -2063,7 +2073,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>70.05</v>
@@ -2122,7 +2132,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>82.955</v>
@@ -2181,7 +2191,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>75.453</v>
@@ -2240,7 +2250,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>72.058</v>
@@ -2299,7 +2309,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>78.697</v>
@@ -2358,7 +2368,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>79.056</v>
@@ -2417,7 +2427,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>72.726</v>
@@ -2476,7 +2486,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>67.312</v>
@@ -2535,7 +2545,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>73.631</v>
@@ -2594,7 +2604,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>81.065</v>
@@ -2653,7 +2663,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>71.81</v>
@@ -2712,7 +2722,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>60.116</v>
@@ -2771,7 +2781,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>70.882</v>
@@ -2830,7 +2840,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>68.268</v>
@@ -2889,7 +2899,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>60.373</v>
@@ -2948,7 +2958,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>65.695</v>
@@ -3007,7 +3017,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>69.771</v>
@@ -3066,7 +3076,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>64.776</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>87.046</v>
@@ -3184,7 +3194,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>79.367</v>
@@ -3243,7 +3253,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>72.42</v>
@@ -3302,7 +3312,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>74.787</v>
@@ -3361,7 +3371,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>67.608</v>
@@ -3420,7 +3430,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>65.8</v>
@@ -3479,7 +3489,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>71.3555</v>
@@ -3538,7 +3548,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>73.692</v>
@@ -3597,7 +3607,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>64.2905</v>
@@ -3656,7 +3666,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>60.527</v>
@@ -3715,7 +3725,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>70.291</v>
@@ -3774,7 +3784,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>72.597</v>
@@ -3833,7 +3843,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>60.973</v>
@@ -3892,7 +3902,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>67.704</v>
@@ -3951,7 +3961,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>77.328</v>
@@ -4010,7 +4020,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>70.704</v>
@@ -4069,7 +4079,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>70.836</v>
@@ -4128,7 +4138,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>65.703</v>
@@ -4187,7 +4197,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>65.884</v>
@@ -4246,7 +4256,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>63.259</v>
@@ -4305,7 +4315,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>55.23</v>
@@ -4364,7 +4374,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>60.865</v>
@@ -4423,7 +4433,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>66.823</v>
@@ -4482,7 +4492,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>66.726</v>
@@ -4541,7 +4551,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>61.185</v>
@@ -4600,7 +4610,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>33.184</v>
@@ -4659,7 +4669,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>75.79</v>
@@ -4718,7 +4728,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>74.809</v>
@@ -4777,7 +4787,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>74.937</v>
@@ -4836,7 +4846,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>83.357</v>
@@ -4895,7 +4905,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>78.522</v>
@@ -4954,7 +4964,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>73.12</v>
@@ -5013,7 +5023,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>76.726</v>
@@ -5072,7 +5082,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>91.187</v>
@@ -5131,7 +5141,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>75.475</v>
@@ -5190,7 +5200,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>82.884</v>
@@ -5249,7 +5259,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>81.745</v>
@@ -5308,7 +5318,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>86.53</v>
@@ -5367,7 +5377,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>87.103</v>
@@ -5426,7 +5436,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>82.518</v>
@@ -5485,7 +5495,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>86.718</v>
@@ -5544,7 +5554,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>86.566</v>
@@ -5603,7 +5613,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>82.84</v>
@@ -5662,7 +5672,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>82.611</v>
@@ -5721,7 +5731,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>79.522</v>
@@ -5780,7 +5790,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>74.938</v>
@@ -5839,7 +5849,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>86.256</v>
@@ -5898,7 +5908,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>86.282</v>
@@ -5957,7 +5967,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2"/>
       <c r="C78" s="3" t="n">
@@ -5990,7 +6000,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2"/>
       <c r="C79" s="3" t="n">
@@ -6023,7 +6033,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2"/>
       <c r="C80" s="3" t="n">
@@ -6056,7 +6066,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2"/>
       <c r="C81" s="3" t="n">
@@ -6089,7 +6099,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="3"/>
@@ -6112,7 +6122,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -6135,7 +6145,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2"/>
       <c r="C84" s="3"/>
@@ -6158,7 +6168,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2"/>
       <c r="C85" s="3"/>
@@ -6181,7 +6191,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2"/>
       <c r="C86" s="3"/>
@@ -6204,7 +6214,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="3"/>
@@ -6227,7 +6237,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2"/>
       <c r="C88" s="3"/>
@@ -6250,7 +6260,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2"/>
       <c r="C89" s="3"/>
@@ -6273,7 +6283,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2"/>
       <c r="C90" s="3"/>
@@ -6296,7 +6306,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
@@ -6319,7 +6329,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="3"/>
@@ -6342,7 +6352,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2"/>
       <c r="C93" s="3"/>
@@ -6365,7 +6375,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
@@ -6388,7 +6398,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2"/>
       <c r="C95" s="3"/>
@@ -6411,7 +6421,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -6434,7 +6444,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="3"/>
@@ -6468,97 +6478,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -6582,7 +6592,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -6592,13 +6602,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.0143909663492046</v>
@@ -6606,7 +6616,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.0549177632913489</v>
@@ -6614,7 +6624,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.00528574400128268</v>
@@ -6622,7 +6632,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.137801449851668</v>
@@ -6630,7 +6640,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.342637246779251</v>
@@ -6638,7 +6648,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.133161196420219</v>
@@ -6646,7 +6656,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.0283701131038142</v>
@@ -6654,7 +6664,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-0.179612555020879</v>
@@ -6662,7 +6672,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>-0.238445213843736</v>

</xml_diff>

<commit_message>
Corrida | GSF-EPRIV-INF | 2026-06-17 11:34:49.319607
</commit_message>
<xml_diff>
--- a/indicadores/GSF-EPRIV-INF_out.xlsx
+++ b/indicadores/GSF-EPRIV-INF_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>